<commit_message>
feat: add post-game recap templates and references for Cyclones and Don't Cha Know teams fix: ensure proper formatting in game log and CSV files style: update season workbook header borders in export functionality test: validate header border styles in league summary sheet
</commit_message>
<xml_diff>
--- a/data/output/stats-fray-late_summer_2026.xlsx
+++ b/data/output/stats-fray-late_summer_2026.xlsx
@@ -824,12 +824,12 @@
           <t>Team OPS</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Through Date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Workbook Season</t>
         </is>

</xml_diff>

<commit_message>
feat: add post-game recap templates and references for Cyclones and Don't Cha Know teams (#25)
fix: ensure proper formatting in game log and CSV files
style: update season workbook header borders in export functionality
test: validate header border styles in league summary sheet
</commit_message>
<xml_diff>
--- a/data/output/stats-fray-late_summer_2026.xlsx
+++ b/data/output/stats-fray-late_summer_2026.xlsx
@@ -824,12 +824,12 @@
           <t>Team OPS</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Through Date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Workbook Season</t>
         </is>

</xml_diff>

<commit_message>
feat: sorting Excel game tabs
</commit_message>
<xml_diff>
--- a/data/output/stats-fray-late_summer_2026.xlsx
+++ b/data/output/stats-fray-late_summer_2026.xlsx
@@ -12,20 +12,20 @@
     <sheet name="Player Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cyclo Total" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cyclo Late Summer 2026 Total" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cyclo Late Summer 2026 Game 1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cyclo Late Summer 2026 Game 2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cyclo Late Summer 2026 Game 3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Cyclo Late Summer 2026 Game 4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Cyclo Late Summer 2026 Game 4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cyclo Late Summer 2026 Game 3" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cyclo Late Summer 2026 Game 2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cyclo Late Summer 2026 Game 1" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$J$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Player Summary'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cyclo Total'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Late Summer 2026 Game 3'!$A$1:$Q$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Late Summer 2026 Game 4'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 4'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 3'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5545,7 +5545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5667,10 +5667,10 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -5694,26 +5694,26 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>0.750</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.250</t>
         </is>
       </c>
     </row>
@@ -5733,16 +5733,16 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -5754,7 +5754,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
         <v>3</v>
@@ -5771,32 +5771,32 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>3.000</t>
+          <t>3.500</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Baxter</t>
+          <t>Bryce</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -5811,42 +5811,42 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.917</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bryce</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -5859,10 +5859,10 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -5880,7 +5880,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
         <v>3</v>
@@ -5897,29 +5897,29 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chance</t>
+          <t>Cory</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -5931,10 +5931,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -5943,49 +5943,49 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M6" t="n">
         <v>2</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.200</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.200</t>
+          <t>1.667</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.533</t>
+          <t>2.334</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cory</t>
+          <t>Erica</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -5994,7 +5994,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -6006,49 +6006,49 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>1.000</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>3.333</t>
-        </is>
-      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4.333</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kyla</t>
+          <t>Kap</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -6069,40 +6069,40 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1.833</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>3</v>
@@ -6111,10 +6111,10 @@
         <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -6126,7 +6126,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -6144,153 +6144,1031 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>1.000</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2.333</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.333</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Stephen</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" t="inlineStr">
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>0.667</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1.667</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2.334</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F12" s="2" t="n">
+      <c r="C13" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F13" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>0.743</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>0.743</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>1.314</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>2.057</t>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.818</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.818</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1.273</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>2.091</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q10"/>
+  <autoFilter ref="A1:Q11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.417</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baxter</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Briana</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.666</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>3.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Erica</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kyla</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rafael</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>3.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
@@ -7231,14 +8109,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7357,16 +8235,16 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -7375,7 +8253,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -7391,7 +8269,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -7401,12 +8279,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.417</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
@@ -7426,13 +8304,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -7447,10 +8325,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -7464,12 +8342,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>3.000</t>
         </is>
       </c>
     </row>
@@ -7480,19 +8358,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -7510,52 +8388,52 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.250</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.917</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Briana</t>
+          <t>Bryce</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -7573,49 +8451,49 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0.666</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bryce</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -7639,26 +8517,26 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.200</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.200</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.533</t>
         </is>
       </c>
     </row>
@@ -7672,25 +8550,25 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -7699,7 +8577,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
         <v>3</v>
@@ -7716,35 +8594,35 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>3.333</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>4.333</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Erica</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -7762,52 +8640,52 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.833</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kyla</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -7816,7 +8694,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -7825,46 +8703,46 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -7876,10 +8754,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -7888,14 +8766,14 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>2</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -7905,958 +8783,80 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.667</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Rafael</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>3</v>
-      </c>
-      <c r="M11" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>2.500</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>3.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+          <t>2.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>1.500</t>
+      <c r="B12" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>0.743</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>0.743</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>1.314</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2.057</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>HRO</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>RBI</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>OBP</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>SLG</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>OPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Alex</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1.250</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Anthony</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2.500</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>3.500</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Bryce</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2.333</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Chance</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cory</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>1.667</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2.334</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Erica</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>1.750</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Kap</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0.333</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0.333</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Kyla</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1.750</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Paul</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2.333</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Stephen</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>1.500</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TEAM TOTALS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>0.818</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>0.818</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>1.273</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>2.091</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:Q11"/>
+  <autoFilter ref="A1:Q10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: sorting Excel game tabs (#27)
</commit_message>
<xml_diff>
--- a/data/output/stats-fray-late_summer_2026.xlsx
+++ b/data/output/stats-fray-late_summer_2026.xlsx
@@ -12,20 +12,20 @@
     <sheet name="Player Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cyclo Total" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cyclo Late Summer 2026 Total" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cyclo Late Summer 2026 Game 1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cyclo Late Summer 2026 Game 2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cyclo Late Summer 2026 Game 3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Cyclo Late Summer 2026 Game 4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Cyclo Late Summer 2026 Game 4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cyclo Late Summer 2026 Game 3" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cyclo Late Summer 2026 Game 2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cyclo Late Summer 2026 Game 1" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$J$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Player Summary'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cyclo Total'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Late Summer 2026 Game 3'!$A$1:$Q$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Late Summer 2026 Game 4'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 4'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 3'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5545,7 +5545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5667,10 +5667,10 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -5694,26 +5694,26 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>0.750</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.250</t>
         </is>
       </c>
     </row>
@@ -5733,16 +5733,16 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -5754,7 +5754,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
         <v>3</v>
@@ -5771,32 +5771,32 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>3.000</t>
+          <t>3.500</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Baxter</t>
+          <t>Bryce</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -5811,42 +5811,42 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.917</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bryce</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -5859,10 +5859,10 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -5880,7 +5880,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
         <v>3</v>
@@ -5897,29 +5897,29 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chance</t>
+          <t>Cory</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -5931,10 +5931,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -5943,49 +5943,49 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M6" t="n">
         <v>2</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.200</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.200</t>
+          <t>1.667</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.533</t>
+          <t>2.334</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cory</t>
+          <t>Erica</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -5994,7 +5994,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -6006,49 +6006,49 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>1.000</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>3.333</t>
-        </is>
-      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4.333</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kyla</t>
+          <t>Kap</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
@@ -6069,40 +6069,40 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1.833</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>3</v>
@@ -6111,10 +6111,10 @@
         <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -6126,7 +6126,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -6144,153 +6144,1031 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>1.000</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2.333</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.333</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Stephen</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" t="n">
-        <v>2</v>
-      </c>
-      <c r="N10" t="inlineStr">
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>0.667</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1.667</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2.334</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B13" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F12" s="2" t="n">
+      <c r="C13" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F13" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>0.743</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>0.743</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>1.314</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>2.057</t>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.818</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.818</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1.273</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>2.091</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q10"/>
+  <autoFilter ref="A1:Q11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.417</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baxter</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Briana</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.666</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>3.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Erica</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kyla</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rafael</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>3.167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
@@ -7231,14 +8109,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7357,16 +8235,16 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -7375,7 +8253,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -7391,7 +8269,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -7401,12 +8279,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.417</t>
+          <t>1.750</t>
         </is>
       </c>
     </row>
@@ -7426,13 +8304,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -7447,10 +8325,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -7464,12 +8342,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>3.000</t>
         </is>
       </c>
     </row>
@@ -7480,19 +8358,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -7510,52 +8388,52 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.250</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.917</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Briana</t>
+          <t>Bryce</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -7573,49 +8451,49 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0.666</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bryce</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -7639,26 +8517,26 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.200</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.200</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.533</t>
         </is>
       </c>
     </row>
@@ -7672,25 +8550,25 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -7699,7 +8577,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
         <v>3</v>
@@ -7716,35 +8594,35 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>3.333</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>4.333</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Erica</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -7762,52 +8640,52 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.833</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kyla</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -7816,7 +8694,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -7825,46 +8703,46 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -7876,10 +8754,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -7888,14 +8766,14 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>2</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -7905,958 +8783,80 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.667</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Rafael</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>3</v>
-      </c>
-      <c r="M11" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>2.500</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>3.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+          <t>2.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>1.500</t>
+      <c r="B12" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>0.743</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>0.743</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>1.314</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2.057</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>AB</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>HRO</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>RBI</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>OBP</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>SLG</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>OPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Alex</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1.250</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Anthony</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2.500</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>3.500</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Bryce</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2.333</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Chance</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cory</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>1.667</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2.334</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Erica</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>1.750</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Kap</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0.333</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0.333</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Kyla</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0.750</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1.750</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Paul</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1.333</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2.333</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Stephen</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0.667</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>1.500</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2.167</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TEAM TOTALS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>0.818</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>0.818</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>1.273</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>2.091</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:Q11"/>
+  <autoFilter ref="A1:Q10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>